<commit_message>
bill counter update check.
</commit_message>
<xml_diff>
--- a/orders/sample_order.xlsx
+++ b/orders/sample_order.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ejasaki\project\python-util\orders\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\crystal-code\python-util\orders\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DDDA95-71C6-4E9C-A9E0-99116C8F6BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="11496"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -37,9 +36,6 @@
     <t>BR0001</t>
   </si>
   <si>
-    <t>Akshat Jain</t>
-  </si>
-  <si>
     <t>BR0006</t>
   </si>
   <si>
@@ -77,12 +73,15 @@
   </si>
   <si>
     <t>dc0002</t>
+  </si>
+  <si>
+    <t>Dr Mehra</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -427,25 +426,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -456,7 +455,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -467,9 +466,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>2</v>
@@ -478,9 +477,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -489,9 +488,9 @@
         <v>310</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>2</v>
@@ -500,9 +499,9 @@
         <v>410</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -511,9 +510,9 @@
         <v>750</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -522,9 +521,9 @@
         <v>310</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>2</v>
@@ -533,9 +532,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -544,9 +543,9 @@
         <v>525</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -555,9 +554,9 @@
         <v>325</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -566,9 +565,9 @@
         <v>450</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -577,9 +576,9 @@
         <v>750</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -588,9 +587,9 @@
         <v>1950</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -599,9 +598,9 @@
         <v>350</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17">
         <v>2</v>

</xml_diff>